<commit_message>
Replace raw numeric exports with unique designer configuration and editable metadata
</commit_message>
<xml_diff>
--- a/config/战场布局.xlsx
+++ b/config/战场布局.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数" sheetId="1" r:id="R3d27b17a7f1b4130"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数" sheetId="1" r:id="R02e43665d1f34eaa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -68,8 +68,12 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -78,13 +82,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Parameters" displayName="Parameters" ref="A1:E13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="5">
-    <x:tableColumn id="1" name="参数ID（勿改）"/>
-    <x:tableColumn id="2" name="对象 / 参数"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Parameters" displayName="Parameters" ref="A1:F11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="所属对象"/>
+    <x:tableColumn id="2" name="字段"/>
     <x:tableColumn id="3" name="配置值（修改此列）"/>
-    <x:tableColumn id="4" name="初始参考值"/>
-    <x:tableColumn id="5" name="来源"/>
+    <x:tableColumn id="4" name="类型"/>
+    <x:tableColumn id="5" name="填写说明"/>
+    <x:tableColumn id="6" name="唯一ID（勿改）"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -285,238 +290,238 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="43" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="70" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="45" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="72" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="68" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="70" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>参数ID（勿改）</x:v>
+        <x:v>所属对象</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>对象 / 参数</x:v>
+        <x:v>字段</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
         <x:v>配置值（修改此列）</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>初始参考值</x:v>
+        <x:v>类型</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>来源</x:v>
+        <x:v>填写说明</x:v>
+      </x:c>
+      <x:c r="F1" s="3" t="str">
+        <x:v>唯一ID（勿改）</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="1" t="str">
-        <x:v>layout.world_length</x:v>
+        <x:v>画面投影</x:v>
       </x:c>
       <x:c r="B2" s="1" t="str">
-        <x:v>显示世界长度</x:v>
-      </x:c>
-      <x:c r="C2" s="5" t="n">
-        <x:v>1800</x:v>
-      </x:c>
-      <x:c r="D2" s="6" t="n">
-        <x:v>1800</x:v>
+        <x:v>屏幕左右留白（像素）</x:v>
+      </x:c>
+      <x:c r="C2" s="6" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="str">
+        <x:v>数值</x:v>
       </x:c>
       <x:c r="E2" s="1" t="str">
-        <x:v>Godot</x:v>
+        <x:v>填写最终生效值</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="str">
+        <x:v>layout.edge_padding</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="1" t="str">
-        <x:v>layout.edge_padding</x:v>
+        <x:v>画面投影</x:v>
       </x:c>
       <x:c r="B3" s="1" t="str">
-        <x:v>屏幕左右留白（像素）</x:v>
-      </x:c>
-      <x:c r="C3" s="5" t="n">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="D3" s="6" t="n">
-        <x:v>18</x:v>
+        <x:v>道路顶边高度比例</x:v>
+      </x:c>
+      <x:c r="C3" s="6" t="n">
+        <x:v>0.69</x:v>
+      </x:c>
+      <x:c r="D3" s="1" t="str">
+        <x:v>数值</x:v>
       </x:c>
       <x:c r="E3" s="1" t="str">
-        <x:v>Godot</x:v>
+        <x:v>填写最终生效值</x:v>
+      </x:c>
+      <x:c r="F3" s="1" t="str">
+        <x:v>layout.road_top</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="1" t="str">
-        <x:v>layout.road_top</x:v>
+        <x:v>画面投影</x:v>
       </x:c>
       <x:c r="B4" s="1" t="str">
-        <x:v>道路顶边占画面高度比例</x:v>
-      </x:c>
-      <x:c r="C4" s="5" t="n">
-        <x:v>0.69</x:v>
-      </x:c>
-      <x:c r="D4" s="6" t="n">
-        <x:v>0.69</x:v>
+        <x:v>道路纵深高度比例</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="n">
+        <x:v>0.21</x:v>
+      </x:c>
+      <x:c r="D4" s="1" t="str">
+        <x:v>数值</x:v>
       </x:c>
       <x:c r="E4" s="1" t="str">
-        <x:v>Godot</x:v>
+        <x:v>填写最终生效值</x:v>
+      </x:c>
+      <x:c r="F4" s="1" t="str">
+        <x:v>layout.road_depth</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="1" t="str">
-        <x:v>layout.road_depth</x:v>
+        <x:v>画面投影</x:v>
       </x:c>
       <x:c r="B5" s="1" t="str">
-        <x:v>道路纵深占画面高度比例</x:v>
-      </x:c>
-      <x:c r="C5" s="5" t="n">
-        <x:v>0.21</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="n">
-        <x:v>0.21</x:v>
+        <x:v>远处尺寸倍率</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="n">
+        <x:v>0.82</x:v>
+      </x:c>
+      <x:c r="D5" s="1" t="str">
+        <x:v>数值</x:v>
       </x:c>
       <x:c r="E5" s="1" t="str">
-        <x:v>Godot</x:v>
+        <x:v>填写最终生效值</x:v>
+      </x:c>
+      <x:c r="F5" s="1" t="str">
+        <x:v>layout.far_scale</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="1" t="str">
-        <x:v>layout.far_scale</x:v>
+        <x:v>画面投影</x:v>
       </x:c>
       <x:c r="B6" s="1" t="str">
-        <x:v>远端缩放倍率</x:v>
-      </x:c>
-      <x:c r="C6" s="5" t="n">
-        <x:v>0.82</x:v>
-      </x:c>
-      <x:c r="D6" s="6" t="n">
-        <x:v>0.82</x:v>
+        <x:v>全局显示尺寸倍率</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D6" s="1" t="str">
+        <x:v>数值</x:v>
       </x:c>
       <x:c r="E6" s="1" t="str">
-        <x:v>Godot</x:v>
+        <x:v>填写最终生效值</x:v>
+      </x:c>
+      <x:c r="F6" s="1" t="str">
+        <x:v>layout.unit_scale</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="1" t="str">
-        <x:v>layout.unit_scale</x:v>
+        <x:v>战场</x:v>
       </x:c>
       <x:c r="B7" s="1" t="str">
-        <x:v>全局显示尺寸倍率</x:v>
-      </x:c>
-      <x:c r="C7" s="5" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D7" s="6" t="n">
-        <x:v>1</x:v>
+        <x:v>战线长度（逻辑与显示共用）</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="n">
+        <x:v>1800</x:v>
+      </x:c>
+      <x:c r="D7" s="1" t="str">
+        <x:v>数值</x:v>
       </x:c>
       <x:c r="E7" s="1" t="str">
-        <x:v>Godot</x:v>
+        <x:v>填写最终生效值</x:v>
+      </x:c>
+      <x:c r="F7" s="1" t="str">
+        <x:v>world.length</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="1" t="str">
-        <x:v>sim:356</x:v>
+        <x:v>基地</x:v>
       </x:c>
       <x:c r="B8" s="1" t="str">
-        <x:v>逻辑战线长度（同步修改显示世界长度）</x:v>
-      </x:c>
-      <x:c r="C8" s="5" t="n">
-        <x:v>1800</x:v>
-      </x:c>
-      <x:c r="D8" s="6" t="n">
-        <x:v>1800</x:v>
+        <x:v>香港基地距左边界</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="n">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="D8" s="1" t="str">
+        <x:v>数值</x:v>
       </x:c>
       <x:c r="E8" s="1" t="str">
-        <x:v>runtime/core/sim.js:12</x:v>
+        <x:v>填写最终生效值</x:v>
+      </x:c>
+      <x:c r="F8" s="1" t="str">
+        <x:v>world.humanMargin</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="1" t="str">
-        <x:v>sim:410</x:v>
+        <x:v>基地</x:v>
       </x:c>
       <x:c r="B9" s="1" t="str">
-        <x:v>香港基地距左边界（世界单位）</x:v>
-      </x:c>
-      <x:c r="C9" s="5" t="n">
+        <x:v>僵尸基地距右边界</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="n">
         <x:v>330</x:v>
       </x:c>
-      <x:c r="D9" s="6" t="n">
-        <x:v>330</x:v>
+      <x:c r="D9" s="1" t="str">
+        <x:v>数值</x:v>
       </x:c>
       <x:c r="E9" s="1" t="str">
-        <x:v>runtime/core/sim.js:13</x:v>
+        <x:v>填写最终生效值</x:v>
+      </x:c>
+      <x:c r="F9" s="1" t="str">
+        <x:v>world.zombieMargin</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="1" t="str">
-        <x:v>sim:465</x:v>
+        <x:v>基地</x:v>
       </x:c>
       <x:c r="B10" s="1" t="str">
-        <x:v>僵尸基地距右边界（世界单位）</x:v>
-      </x:c>
-      <x:c r="C10" s="5" t="n">
-        <x:v>330</x:v>
-      </x:c>
-      <x:c r="D10" s="6" t="n">
-        <x:v>330</x:v>
+        <x:v>同阵营基地横向间距</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D10" s="1" t="str">
+        <x:v>数值</x:v>
       </x:c>
       <x:c r="E10" s="1" t="str">
-        <x:v>runtime/core/sim.js:14</x:v>
+        <x:v>填写最终生效值</x:v>
+      </x:c>
+      <x:c r="F10" s="1" t="str">
+        <x:v>world.baseSpacing</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="1" t="str">
-        <x:v>sim:571</x:v>
+        <x:v>出兵</x:v>
       </x:c>
       <x:c r="B11" s="1" t="str">
-        <x:v>士兵出生点距基地后方（世界单位）</x:v>
-      </x:c>
-      <x:c r="C11" s="5" t="n">
+        <x:v>出兵点位于基地后方的距离</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="n">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="D11" s="6" t="n">
-        <x:v>78</x:v>
+      <x:c r="D11" s="1" t="str">
+        <x:v>数值</x:v>
       </x:c>
       <x:c r="E11" s="1" t="str">
-        <x:v>runtime/core/sim.js:17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="1" t="str">
-        <x:v>sim:2340</x:v>
-      </x:c>
-      <x:c r="B12" s="1" t="str">
-        <x:v>同阵营基地横向间隔（两侧分别设置）</x:v>
-      </x:c>
-      <x:c r="C12" s="5" t="n">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="D12" s="6" t="n">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="E12" s="1" t="str">
-        <x:v>runtime/core/sim.js:69</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="1" t="str">
-        <x:v>sim:2370</x:v>
-      </x:c>
-      <x:c r="B13" s="1" t="str">
-        <x:v>同阵营基地横向间隔（两侧分别设置）</x:v>
-      </x:c>
-      <x:c r="C13" s="5" t="n">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="D13" s="6" t="n">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="E13" s="1" t="str">
-        <x:v>runtime/core/sim.js:70</x:v>
+        <x:v>填写最终生效值</x:v>
+      </x:c>
+      <x:c r="F11" s="1" t="str">
+        <x:v>world.spawnOffset</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba1665c92a244757"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebff208c57714bf3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>